<commit_message>
v1.1: Dashboard con login, Seguridad (roles), Actualizar base, flujo por mes, gráfico G/P, docs y Vercel
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>14:15</v>
+        <v>16:45</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -444,16 +444,33 @@
         <v>Setup</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>16:45</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Despliegue v1.1</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Dashboard con login, Seguridad (roles), Actualizar base, flujo por mes, gráfico G/P. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -499,9 +516,17 @@
         <v>Carpetas sql/, scripts/, docs/, Base/. Reglas en .cursor/rules (estructura-proyecto, reglas-everfit, bitácora, preguntas-solo-respuesta).</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Dashboard Everfit</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -571,7 +596,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -600,9 +625,20 @@
         <v>Setup: estructura repo, reglas, script bitácora, volcado Excel a Supabase, tipos de cambio por API.</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>1.1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dashboard completo: login por email, módulo Seguridad (roles Admin/Encargado/Visor), Actualizar base (upload Excel), flujo por mes, gráfico G/P, filtros. Despliegue Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.2: config desde env en Vercel, outputDirectory, favicon EF, script vercel-setup-env, docs
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:45</v>
+        <v>17:19</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:45</v>
+        <v>17:19</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -461,9 +461,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>17:19</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Despliegue v1.2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Config desde env en Vercel, outputDirectory, favicon EF, script vercel-setup-env, docs. Push a main.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -596,7 +613,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -636,9 +653,20 @@
         <v>Dashboard completo: login por email, módulo Seguridad (roles Admin/Encargado/Visor), Actualizar base (upload Excel), flujo por mes, gráfico G/P, filtros. Despliegue Vercel.</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1.2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Config build para Vercel (config.js desde env), outputDirectory, favicon EF (logo reducido), script vercel-setup-env, docs URL y dominio.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.3: Proyección Flujo por mes, total con proyectados, tarjetas reales, fondo encabezado proyectados
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>17:19</v>
+        <v>18:14</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>17:19</v>
+        <v>18:14</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>17:19</v>
+        <v>18:14</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -478,16 +478,33 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>18:14</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Despliegue v1.3</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Proyección en Flujo por mes (config, ventana móvil), total tabla con proyectados, tarjetas solo reales, encabezado con fondo en columnas proyectadas.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -541,9 +558,17 @@
         <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador.</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Proyección Flujo por mes</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Meses proyectados en tabla (permiso ver_proyeccion). Config: método (promedio/mediana/promedio recortado), meses de historia, meses a proyectar, recorte %. Ventana móvil. Total columna incluye proyectados; tarjetas siempre reales. Encabezado y celdas proyectadas con fondo distintivo.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -613,7 +638,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -664,9 +689,20 @@
         <v>Config build para Vercel (config.js desde env), outputDirectory, favicon EF (logo reducido), script vercel-setup-env, docs URL y dominio.</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>1.3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Proyección en Flujo por mes: config (método, meses historia, meses a proyectar, recorte %), ventana móvil. Total tabla con proyectados; tarjetas solo reales. Fondo distintivo en encabezado y celdas proyectadas.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.4: Seguridad permisos por rol editables (iconos y toggles on/off)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:14</v>
+        <v>18:26</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:14</v>
+        <v>18:26</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:14</v>
+        <v>18:26</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:14</v>
+        <v>18:26</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -495,16 +495,33 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>18:26</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Despliegue v1.4</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Seguridad: permisos por rol configurables (Admin, Encargado, Visor) con icono y toggles on/off. SQL supabase_seguridad_permisos_editable.sql.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -566,9 +583,17 @@
         <v>Meses proyectados en tabla (permiso ver_proyeccion). Config: método (promedio/mediana/promedio recortado), meses de historia, meses a proyectar, recorte %. Ventana móvil. Total columna incluye proyectados; tarjetas siempre reales. Encabezado y celdas proyectadas con fondo distintivo.</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Seguridad – Permisos por rol</v>
+      </c>
+      <c r="B8" t="str">
+        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Visor) con icono y lista de permisos con toggle on/off editable. RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -638,7 +663,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -700,9 +725,20 @@
         <v>Proyección en Flujo por mes: config (método, meses historia, meses a proyectar, recorte %), ventana móvil. Total tabla con proyectados; tarjetas solo reales. Fondo distintivo en encabezado y celdas proyectadas.</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>1.4</v>
+      </c>
+      <c r="B6" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Seguridad: permisos por rol editables (iconos y toggles on/off para Admin, Encargado, Visor). SQL supabase_seguridad_permisos_editable.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.5: Botón refresh y auto-refresh al cambiar permisos en Seguridad
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:26</v>
+        <v>18:35</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:26</v>
+        <v>18:35</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:26</v>
+        <v>18:35</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:26</v>
+        <v>18:35</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:26</v>
+        <v>18:35</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -512,9 +512,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>18:35</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Despliegue v1.5</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Botón refresh en barra (actualizar permisos y vista sin cerrar sesión). Auto-refresh al cambiar permisos en Seguridad.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -663,7 +680,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -736,9 +753,20 @@
         <v>Seguridad: permisos por rol editables (iconos y toggles on/off para Admin, Encargado, Visor). SQL supabase_seguridad_permisos_editable.sql.</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>1.5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Botón refresh en barra (actualizar permisos y vista sin cerrar sesión). Auto-refresh al cambiar permisos en Seguridad.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.6: Incluir proyectado, help exclusiones, tarjetas en card, config proyección por usuario
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:35</v>
+        <v>20:03</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:35</v>
+        <v>20:03</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:35</v>
+        <v>20:03</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:35</v>
+        <v>20:03</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:35</v>
+        <v>20:03</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:35</v>
+        <v>20:03</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -529,9 +529,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>20:03</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Despliegue v1.6</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Incluir proyectado en tarjetas, gráfico y flujo. Help (?) con reglas de exclusión en los tres. Tarjetas en una card con help dentro. Config proyección por usuario (config_dashboard). Exclusión Dividendos solo tabla.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -680,7 +697,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -764,9 +781,20 @@
         <v>Botón refresh en barra (actualizar permisos y vista sin cerrar sesión). Auto-refresh al cambiar permisos en Seguridad.</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>1.6</v>
+      </c>
+      <c r="B8" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Incluir real_pendiente=proyectado en todo. Help (?) con reglas de exclusión en tarjetas, gráfico y flujo. Tarjetas en una card con help dentro. Config proyección por usuario (config_dashboard). Dividendos solo excluido en tabla.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.7: Gráfico G/P Mensual sin leyenda
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>20:03</v>
+        <v>20:45</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -546,9 +546,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>20:45</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Despliegue v1.7</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Gráfico G/P Mensual: ocultar leyenda (barras verdes/rojas sin leyenda engañosa).</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -697,7 +714,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -792,9 +809,20 @@
         <v>Incluir real_pendiente=proyectado en todo. Help (?) con reglas de exclusión en tarjetas, gráfico y flujo. Tarjetas en una card con help dentro. Config proyección por usuario (config_dashboard). Dividendos solo excluido en tabla.</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>1.7</v>
+      </c>
+      <c r="B9" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Gráfico G/P Mensual: leyenda oculta (barras verdes/rojas sin leyenda).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.8: Gráfico G/P barras G/P=0 visibles (minBarLength, gris, tooltip)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>06/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>20:45</v>
+        <v>21:11</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -563,9 +563,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>21:11</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Despliegue v1.8</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Gráfico G/P: barras con G/P=0 visibles (minBarLength, color gris, tooltip "ingresos = egresos").</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -714,7 +731,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -820,9 +837,20 @@
         <v>Gráfico G/P Mensual: leyenda oculta (barras verdes/rojas sin leyenda).</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>1.8</v>
+      </c>
+      <c r="B10" t="str">
+        <v>06/03/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Gráfico G/P: barras con G/P=0 visibles (minBarLength, color gris, tooltip ingresos=egresos).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.9: Tipos de cambio por API desde origen (Opción 2). Fix upload Excel fechas. ORIGEN_TC_* en config y build.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>06/03/2026</v>
+        <v>07/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>21:11</v>
+        <v>09:30</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -580,9 +580,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Despliegue v1.9</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Tipos de cambio por API desde Sistema-Contable-Nuevo (Opción 2). Fix upload Excel: fechas como ISO. ORIGEN_TC_* en config y build.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -731,7 +748,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -848,9 +865,20 @@
         <v>Gráfico G/P: barras con G/P=0 visibles (minBarLength, color gris, tooltip ingresos=egresos).</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>1.9</v>
+      </c>
+      <c r="B11" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Tipos de cambio por API desde Sistema-Contable-Nuevo (Opción 2). Fix upload Excel fechas→ISO. ORIGEN_TC_* en config y build.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.10: Modal gráfico por ítem en detalle e icono en totales, icono sin contorno, sucursales turquesa
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>09:30</v>
+        <v>10:55</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -597,9 +597,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>10:55</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Despliegue v1.10</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Modal gráfico por ítem en detalle (concepto/beneficiario) e icono en totales (Ingresos, Egresos, G/P). Icono sin contorno. Botones sucursal seleccionado en turquesa (#0d9488).</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -748,7 +765,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -870,15 +887,26 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>07/03/2026</v>
+        <v>06/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Tipos de cambio por API desde Sistema-Contable-Nuevo (Opción 2). Fix upload Excel fechas→ISO. ORIGEN_TC_* en config y build.</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>1.10</v>
+      </c>
+      <c r="B12" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Modal gráfico por ítem en detalle (concepto/beneficiario) e icono en totales. Icono sin contorno. Botones sucursal seleccionado en turquesa.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.11: Log actualización base, leyenda Última actualización, progreso eliminación en upload, fix RPC
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>10:55</v>
+        <v>12:51</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -614,9 +614,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>12:51</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Despliegue v1.11</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Log actualización base (tabla, RPC, leyenda Última actualización con reloj y hora Argentina). Progreso eliminación en upload (Eliminando X / N). Fix RPC sin .catch.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -765,7 +782,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -904,9 +921,20 @@
         <v>Modal gráfico por ítem en detalle (concepto/beneficiario) e icono en totales. Icono sin contorno. Botones sucursal seleccionado en turquesa.</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>1.11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Log actualización base y leyenda Última actualización. Progreso eliminación en upload. Fix RPC log.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.12: Dashboard responsive móviles, regla responsive en reglas-everfit
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>07/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:51</v>
+        <v>13:13</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -631,9 +631,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>13:13</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Despliegue v1.12</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Dashboard responsive para móviles (breakpoints 768px y 480px, touch 44px, safe-area, tablas y modales adaptados). Regla responsive en reglas-everfit.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -782,7 +799,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -932,9 +949,20 @@
         <v>Log actualización base y leyenda Última actualización. Progreso eliminación en upload. Fix RPC log.</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>1.12</v>
+      </c>
+      <c r="B14" t="str">
+        <v>07/03/2026</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Dashboard responsive móviles. Regla: tener en cuenta responsive a partir de ahora.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.13: Filtro multi-sucursal, sucursales por usuario en Seguridad, Total respeta asignación
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>07/03/2026</v>
+        <v>08/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:13</v>
+        <v>13:32</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -648,9 +648,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>08/03/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>13:32</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Despliegue v1.13</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Filtro multi-sucursal (varias sucursales a la vez). Seguridad: sucursales permitidas por usuario (Admin configura qué ve cada uno). Total respeta sucursales asignadas. SQL supabase_sucursales_por_usuario.sql.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -799,7 +816,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -960,9 +977,20 @@
         <v>Dashboard responsive móviles. Regla: tener en cuenta responsive a partir de ahora.</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>1.13</v>
+      </c>
+      <c r="B15" t="str">
+        <v>08/03/2026</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.14: modales backdrop real click (setupBackdropCloseOnlyOnRealClick)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:32</v>
+        <v>18:12</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -665,9 +665,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>18:12</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Despliegue v1.14</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -816,7 +833,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -982,15 +999,26 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>08/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>1.14</v>
+      </c>
+      <c r="B16" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.15: paginación tipos de cambio, regla PostgREST y despliegue
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:12</v>
+        <v>18:07</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -682,9 +682,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Despliegue v1.15</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Tipos de cambio cargados con paginación (límite PostgREST ~1000 filas por consulta). Constante SUPABASE_PAGE_SIZE alineada con base_everfit. Regla reglas-everfit actualizada. Despliegue a producción.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -742,7 +759,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador.</v>
+        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador. Carga paginada de base_everfit y de tipos de cambio (evita tope ~1000 filas de PostgREST).</v>
       </c>
     </row>
     <row r="7">
@@ -833,7 +850,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -999,7 +1016,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
@@ -1010,15 +1027,26 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1.15</v>
+      </c>
+      <c r="B17" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Tipos de cambio con paginación al cargar (tipos_cambio_global / tipo_de_cambio). Regla proyecto: documentar límite PostgREST y paginación en reglas-everfit.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.16: fechas Argentina en gráfico G/P y agrupación fecha_pago ISO
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -684,10 +684,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>18:07</v>
+        <v>08:55</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -699,9 +699,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>08:55</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Dashboard fechas Argentina</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Gráfico G/P mensual y proyección: mes actual con calendario Argentina (no zona del navegador). fecha_pago ISO/timestamptz: agrupar por día en Argentina (evita slice UTC).</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>08:55</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Despliegue v1.16</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Fechas Argentina en gráfico G/P (rango 13 meses y mes en curso/proyección) y agrupación por día calendario en fecha_pago con hora desde Supabase. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -759,7 +793,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador. Carga paginada de base_everfit y de tipos de cambio (evita tope ~1000 filas de PostgREST).</v>
+        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Fechas de negocio y mes actual en America/Argentina/Buenos_Aires (incl. fecha_pago con hora desde Supabase). Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador. Carga paginada de base_everfit y de tipos de cambio (evita tope ~1000 filas de PostgREST).</v>
       </c>
     </row>
     <row r="7">
@@ -850,7 +884,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1016,7 +1050,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
@@ -1027,7 +1061,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -1038,15 +1072,26 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>19/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Tipos de cambio con paginación al cargar (tipos_cambio_global / tipo_de_cambio). Regla proyecto: documentar límite PostgREST y paginación en reglas-everfit.</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>1.16</v>
+      </c>
+      <c r="B18" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Fechas America/Argentina/Buenos_Aires: gráfico G/P y clave mes en curso; fecha_pago ISO/timestamptz agrupada por día local (no slice UTC).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.17: gráfico G/P alineado con tabla Flujo (excluye Dividendos)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>08:55</v>
+        <v>08:59</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -733,9 +733,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>08:59</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Despliegue v1.17</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Gráfico G/P Mensual usa porMesFlujo: mismos totales por mes que la tabla Flujo (excluye Dividendos). Ayuda (?), pie de tabla y docs/EXCLUSIONES_DASHBOARD.md.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -793,7 +810,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P, filtros moneda/sucursal. Fechas de negocio y mes actual en America/Argentina/Buenos_Aires (incl. fecha_pago con hora desde Supabase). Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador. Carga paginada de base_everfit y de tipos de cambio (evita tope ~1000 filas de PostgREST).</v>
+        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P (mismos totales por mes que la tabla Flujo; excluye Dividendos), filtros moneda/sucursal. Fechas de negocio y mes actual en America/Argentina/Buenos_Aires (incl. fecha_pago con hora desde Supabase). Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador. Carga paginada de base_everfit y de tipos de cambio (evita tope ~1000 filas de PostgREST).</v>
       </c>
     </row>
     <row r="7">
@@ -884,7 +901,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1089,9 +1106,20 @@
         <v>Fechas America/Argentina/Buenos_Aires: gráfico G/P y clave mes en curso; fecha_pago ISO/timestamptz agrupada por día local (no slice UTC).</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>1.17</v>
+      </c>
+      <c r="B19" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Gráfico G/P Mensual alineado con tabla Flujo por mes (porMesFlujo; excluye Dividendos). Documentación EXCLUSIONES_DASHBOARD.md actualizada.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.18: fechas AR, gráfico alineado con Flujo, tarjetas con Dividendos, UX local
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>31/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>08:59</v>
+        <v>09:10</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -750,9 +750,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>09:10</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Dashboard local: mensaje si falta config</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Mensaje visible fuera de app-content cuando falta SUPABASE_ANON_KEY (config.js en .gitignore). Errores RPC/sesión muestran panel en la app en lugar de pantalla en blanco.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>09:10</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Tarjetas: otra vez con Dividendos</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Cards vuelven a porMes (incluyen Dividendos); tabla y gráfico siguen con porMesFlujo. Criterio documentado en EXCLUSIONES_DASHBOARD.md.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>09:10</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Despliegue v1.18</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Fechas Argentina en fecha_pago y rango G/P; gráfico alineado con tabla Flujo (porMesFlujo); tarjetas con porMes (incluye Dividendos); mensaje si falta config local; manejo errores RPC/sesión; docs EXCLUSIONES. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -810,7 +861,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes, resumen, gráfico G/P (mismos totales por mes que la tabla Flujo; excluye Dividendos), filtros moneda/sucursal. Fechas de negocio y mes actual en America/Argentina/Buenos_Aires (incl. fecha_pago con hora desde Supabase). Login por email; módulo Seguridad (Admin asigna roles). Actualizar base: truncar y cargar Excel desde el navegador. Carga paginada de base_everfit y de tipos de cambio (evita tope ~1000 filas de PostgREST).</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Fechas en America/Argentina/Buenos_Aires. Login por email; Seguridad; actualizar base desde el navegador. Carga paginada de base_everfit y tipos de cambio.</v>
       </c>
     </row>
     <row r="7">
@@ -901,7 +952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1117,9 +1168,20 @@
         <v>Gráfico G/P Mensual alineado con tabla Flujo por mes (porMesFlujo; excluye Dividendos). Documentación EXCLUSIONES_DASHBOARD.md actualizada.</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="B20" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Consolidado: fechas AR en agrupación y mes actual; gráfico=tabla Flujo; tarjetas con Dividendos; UX local sin anon key y errores sesión/RPC visibles. EXCLUSIONES_DASHBOARD.md.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: tabla transacciones_asistencia e import Excel por sucursal desde dashboard
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -684,10 +684,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -701,10 +701,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -718,10 +718,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -735,10 +735,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -752,10 +752,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -769,10 +769,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -786,10 +786,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>09:10</v>
+        <v>09:58</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -801,16 +801,33 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>09:58</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Transacciones asistencia → Supabase</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Tabla transacciones_asistencia (sql/), import Excel Sheet1 desde dashboard (Importar asistencia, permiso upload_base). Normaliza Cramer/Cabildo/Migueletes. Docs TRANSACCIONES_ASISTENCIA.md.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -861,7 +878,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Fechas en America/Argentina/Buenos_Aires. Login por email; Seguridad; actualizar base desde el navegador. Carga paginada de base_everfit y tipos de cambio.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel Transacciones por sucursal → transacciones_asistencia). Fechas en America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit y tipos de cambio.</v>
       </c>
     </row>
     <row r="7">
@@ -880,9 +897,17 @@
         <v>En Seguridad (Admin): cada rol (Admin, Encargado, Visor) con icono y lista de permisos con toggle on/off editable. RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql.</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Transacciones de asistencia</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Excel export Transacciones por sucursal (docs de referencia). Tabla transacciones_asistencia; botón Importar asistencia en dashboard (reemplazo por sucursal). Ver docs/TRANSACCIONES_ASISTENCIA.md y sql/supabase_transacciones_asistencia.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1118,7 +1143,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
@@ -1129,7 +1154,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -1140,7 +1165,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Tipos de cambio con paginación al cargar (tipos_cambio_global / tipo_de_cambio). Regla proyecto: documentar límite PostgREST y paginación en reglas-everfit.</v>
@@ -1151,7 +1176,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Fechas America/Argentina/Buenos_Aires: gráfico G/P y clave mes en curso; fecha_pago ISO/timestamptz agrupada por día local (no slice UTC).</v>
@@ -1162,7 +1187,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Gráfico G/P Mensual alineado con tabla Flujo por mes (porMesFlujo; excluye Dividendos). Documentación EXCLUSIONES_DASHBOARD.md actualizada.</v>
@@ -1173,7 +1198,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>31/03/2026</v>
+        <v>16/04/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Consolidado: fechas AR en agrupación y mes actual; gráfico=tabla Flujo; tarjetas con Dividendos; UX local sin anon key y errores sesión/RPC visibles. EXCLUSIONES_DASHBOARD.md.</v>

</xml_diff>

<commit_message>
v1.19: vista Asistencia (heatmap, permiso ver_asistencia, SQL y docs)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>09:58</v>
+        <v>11:08</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -818,9 +818,94 @@
         <v>Feature</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>11:08</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Menú Asistencia en dashboard</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Vista Asistencia: heatmap concurrencia por día y hora (1 h por ingreso), año y mes o todos los meses, franja horaria, filtro multi-sucursal y permisos; clientes en más de una sede; carga paginada; índice (fecha, sucursal); invalidación de caché al importar.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>11:08</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Combo año Asistencia desde datos</v>
+      </c>
+      <c r="D26" t="str">
+        <v>RPC get_anios_transacciones_asistencia: el select de año solo lista años con registros en transacciones_asistencia; fallback año actual si tabla vacía o RPC no ejecutada.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>11:08</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Tabla multi-sede Asistencia</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Visitas por sede con conteo por cliente; resaltado ámbar la(s) sede(s) con más visitas (empate).</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>11:08</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Permiso ver_asistencia</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Menú Asistencia y SELECT transacciones_asistencia condicionados a ver_asistencia; toggles en Seguridad; sql/supabase_asistencia_ver_permiso.sql y DDL transacciones actualizado.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>11:08</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Despliegue v1.19</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Vista Asistencia: heatmap verde-rojo, franja horaria, filas calendario o Lun–Dom, combo años RPC, carga y mapa por fecha optimizado, multi-sede con visitas por sede y filtro una sucursal; ver_asistencia; mensajes al filtrar. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -878,7 +963,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel Transacciones por sucursal → transacciones_asistencia). Fechas en America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit y tipos de cambio.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC), multi-sede y tabla por sede. Fechas en America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -894,7 +979,7 @@
         <v>Seguridad – Permisos por rol</v>
       </c>
       <c r="B8" t="str">
-        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Visor) con icono y lista de permisos con toggle on/off editable. RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql.</v>
+        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Visor) con icono y lista de permisos con toggle on/off editable (incluye ver_asistencia para el menú Asistencia). RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql y sql/supabase_asistencia_ver_permiso.sql si aplica.</v>
       </c>
     </row>
     <row r="9">
@@ -977,7 +1062,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1204,9 +1289,20 @@
         <v>Consolidado: fechas AR en agrupación y mes actual; gráfico=tabla Flujo; tarjetas con Dividendos; UX local sin anon key y errores sesión/RPC visibles. EXCLUSIONES_DASHBOARD.md.</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>1.19</v>
+      </c>
+      <c r="B21" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Asistencia: menú y permiso ver_asistencia (RLS, sql migración); heatmap por franja horaria, modo filas calendario o Lun–Dom, años vía RPC, optimización índice por fecha y caché; multi-sede con conteos por sede y lógica filtro una sede; UX carga filtros; índice (fecha,sucursal) en DDL.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.20: Asistencia frecuencia por semanas activas y despliegue
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>11:08</v>
+        <v>11:55</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -903,9 +903,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>11:55</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Asistencia: frecuencia de uso</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Distribución por rangos: días distintos con visita ÷ semanas (lun–dom) con ≥1 ingreso (no diluye meses sin asistir). Sin tramo «menos de 1 día/sem» (mínimo 1 con semanas activas). Multi-sede: prom. ingr./sem. activas.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>11:55</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Despliegue v1.20</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Asistencia: frecuencia por semanas activas (lun–dom con ingreso); distribución por rangos desde 1 día/sem.; multi-sede con prom. ingr./sem. activas; textos de ayuda. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -963,7 +997,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC), multi-sede y tabla por sede. Fechas en America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC), distribución de frecuencia (días distintos ÷ semanas lun–dom con ingreso mientras el cliente activo; tramos desde 1 día/sem., % y rango modal), multi-sede con prom. ingr./sem. activas. Fechas en America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1062,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1300,9 +1334,20 @@
         <v>Asistencia: menú y permiso ver_asistencia (RLS, sql migración); heatmap por franja horaria, modo filas calendario o Lun–Dom, años vía RPC, optimización índice por fecha y caché; multi-sede con conteos por sede y lógica filtro una sede; UX carga filtros; índice (fecha,sucursal) en DDL.</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1.20</v>
+      </c>
+      <c r="B22" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Asistencia frecuencia: distribución por rangos con días distintos ÷ semanas activas (lun–dom con ingreso); sin tramo &lt;1 día/sem.; prom. ingr./sem. activas en multi-sede; textos de ayuda.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.21: Asistencia con progreso de carga, modal nueva versión y SQL índice covering opcional
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E37"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>11:55</v>
+        <v>12:49</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -937,9 +937,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Asistencia: permanencia</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Distribución por meses entre primera y última visita; tramos mensuales 0–12 y cola dinámica hasta 60 meses; promedio global; ayuda (?).</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Asistencia: permanencia aclaración</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Texto y subtítulo: permanencia solo dentro del rango Año/Mes cargado (techo = duración del período); wrap sin max-height para ver tramo 0–1 mes; ayuda (?).</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B34" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Asistencia: filtros y rendimiento</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Clic sucursales con delegación única y detección de vista activa por menú (no display:none). Doble rAF en carga; mapa primero y métricas en siguiente frame. Rango «Todos los años» (min–max años con datos). Al entrar Asistencia o abrir Importar: mes Todos y año Todos si existe opción; modal dispara carga de años si faltan. invalidateAsistenciaCache limpia asistenciaAniosDisponibles. Tras import, refresco si el menú Asistencia está activo.</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B35" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Asistencia: UX carga y SQL índice</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Bajo filtros: bloque de contenido oculto hasta tener datos; modal con spinner y barra (conteo exact PostgREST + progreso por páginas; indeterminada si falla el count). Fase «Armando mapa» con doble rAF. Aviso si &gt;250k filas. sql/supabase_transacciones_asistencia_index_covering.sql (INCLUDE). Docs TRANSACCIONES.</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B36" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Nueva versión Everfit (como Pandi)</v>
+      </c>
+      <c r="D36" t="str">
+        <v>everfit-release.json en raíz + modal al detectar despliegue (fetch no-store); reglas bitacora-tareas y reglas-everfit; docs GIT_Y_VERCEL; estructura-proyecto. Criterio lines comerciales solo lo visible.</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B37" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Despliegue v1.21</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Asistencia: carga con modal de progreso, bloque bajo filtros en blanco hasta tener datos, conteo y paginación; modal «Nueva versión» con everfit-release.json; script índice covering opcional; reglas y docs. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -997,7 +1099,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC), distribución de frecuencia (días distintos ÷ semanas lun–dom con ingreso mientras el cliente activo; tramos desde 1 día/sem., % y rango modal), multi-sede con prom. ingr./sem. activas. Fechas en America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), permanencia acotada al rango, multi-sede. Tras un despliegue: modal «Nueva versión» leyendo **everfit-release.json** (mismo criterio comercial que Pandi; ver bitácora-tareas). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1096,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1345,9 +1447,20 @@
         <v>Asistencia frecuencia: distribución por rangos con días distintos ÷ semanas activas (lun–dom con ingreso); sin tramo &lt;1 día/sem.; prom. ingr./sem. activas en multi-sede; textos de ayuda.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1.21</v>
+      </c>
+      <c r="B23" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Asistencia: UX de carga (modal spinner y barra, área bajo filtros oculta hasta listo, progreso por descarga); aviso de muchos registros; modal «Nueva versión» con everfit-release.json (criterio Pandi); sql índice covering opcional; reglas bitácora y GIT_Y_VERCEL.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.22: permanencia por rango en Asistencia y despliegue
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E40"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -942,7 +942,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -959,7 +959,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -976,7 +976,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -993,7 +993,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1010,7 +1010,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1027,7 +1027,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>12:49</v>
+        <v>13:16</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1039,9 +1039,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B38" t="str">
+        <v>13:16</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Asistencia: detalle permanencia por cliente</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Tabla detalle con acción (ojo): modal con meses de carrera, días distintos, ingresos, tiempo estimado en club (1 h por ingreso); segundo ojito muestra u oculta asistencias ordenadas por fecha y hora.</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B39" t="str">
+        <v>13:16</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Asistencia: permanencia ojo por rango</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Ojo en cada fila de la tabla de rangos (columna Acción a la derecha del %): modal con clientes solo de ese bucket; ojo por cliente con «Volver al listado del rango»; delegación document para clics dentro del modal. Eliminada la tabla global «Detalle por cliente». Ayuda (?), card Permanencia y help-asistencia.</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B40" t="str">
+        <v>13:16</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Despliegue v1.22</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Permanencia por rango en Asistencia, everfit-release.json y sidebar v1.22. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1099,7 +1150,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), permanencia acotada al rango, multi-sede. Tras un despliegue: modal «Nueva versión» leyendo **everfit-release.json** (mismo criterio comercial que Pandi; ver bitácora-tareas). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), **permanencia** acotada al rango: tabla de distribución con columna Acción (ojo por rango) que abre el listado de clientes de ese tramo; desde ahí ojo por cliente (volver al rango) y segundo ojito para asistencias por fecha/hora; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1198,7 +1249,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1458,9 +1509,20 @@
         <v>Asistencia: UX de carga (modal spinner y barra, área bajo filtros oculta hasta listo, progreso por descarga); aviso de muchos registros; modal «Nueva versión» con everfit-release.json (criterio Pandi); sql índice covering opcional; reglas bitácora y GIT_Y_VERCEL.</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1.22</v>
+      </c>
+      <c r="B24" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Asistencia permanencia: columna Acción (ojo) por fila de rango abre modal con clientes de ese bucket; volver al rango desde el detalle; delegación de clics en document; sin tabla global detalle. everfit-release.json v1.22.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Se incorpora el apellido y nombre del cliente en el detalle de permanencia por cliente.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -942,7 +942,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -959,7 +959,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -976,7 +976,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -993,7 +993,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1010,7 +1010,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1027,7 +1027,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1044,7 +1044,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1061,7 +1061,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1078,7 +1078,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>13:16</v>
+        <v>13:22</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1090,9 +1090,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B41" t="str">
+        <v>13:22</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Despliegue v1.23</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Se incorpora el apellido y nombre del cliente en el detalle de permanencia por cliente. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1150,7 +1167,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), **permanencia** acotada al rango: tabla de distribución con columna Acción (ojo por rango) que abre el listado de clientes de ese tramo; desde ahí ojo por cliente (volver al rango) y segundo ojito para asistencias por fecha/hora; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), **permanencia** acotada al rango: tabla de distribución con columna Acción (ojo por rango) que abre el listado de clientes de ese tramo; desde ahí ojo por cliente (volver al rango) y segundo ojito para asistencias por fecha/hora; **modal detalle permanencia: título con apellido y nombre** (junto al ID si aplica) cuando los datos lo permiten; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1249,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1520,9 +1537,20 @@
         <v>Asistencia permanencia: columna Acción (ojo) por fila de rango abre modal con clientes de ese bucket; volver al rango desde el detalle; delegación de clics en document; sin tabla global detalle. everfit-release.json v1.22.</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>1.23</v>
+      </c>
+      <c r="B25" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Se incorpora el apellido y nombre del cliente en el detalle de permanencia por cliente.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.24: Asistencia cache, huella RPC, modal permanencia y sub-rango en memoria
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E46"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -942,7 +942,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -959,7 +959,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -976,7 +976,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -993,7 +993,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1010,7 +1010,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1027,7 +1027,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1044,7 +1044,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1061,7 +1061,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1078,7 +1078,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1095,7 +1095,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>13:22</v>
+        <v>14:03</v>
       </c>
       <c r="C41" t="str">
         <v>Despliegue v1.23</v>
@@ -1107,9 +1107,94 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B42" t="str">
+        <v>14:03</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Asistencia: huella RPC y cache</v>
+      </c>
+      <c r="D42" t="str">
+        <v>RPC get_asistencia_dataset_version(desde,hasta) + comparación antes de re-paginar; invalidación al importar. sql/supabase_asistencia_dataset_version.sql y docs TRANSACCIONES.</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B43" t="str">
+        <v>14:03</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Asistencia: refresh barra sin invalidar cache</v>
+      </c>
+      <c r="D43" t="str">
+        <v>refreshPermisosYVista ya no llama invalidateAsistenciaCache; tras cargarDatos repinta Asistencia si está activa para respetar huella y evitar re-descarga completa.</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B44" t="str">
+        <v>14:03</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Asistencia: nombre en modal por rango</v>
+      </c>
+      <c r="D44" t="str">
+        <v>asistenciaPersonaHtmlLabelPerm muestra ID — Apellido, Nombre cuando hay empleado_id y datos de nombre (tabla Clientes del modal por bucket).</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B45" t="str">
+        <v>14:03</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Asistencia: sub-rango en memoria</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Si el combo Año/Mes pide un rango contenido en el ya descargado (p. ej. 2026 dentro de «todos los años»), no se re-pagina Supabase; filtro por fecha en getAsistenciaRowsFiltered. Huella RPC solo si UI = rango del cache.</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B46" t="str">
+        <v>14:03</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Despliegue v1.24</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Asistencia: huella RPC, cache/refresh, sub-rango en memoria, modal permanencia por rango (layout + nombres). sql supabase_asistencia_dataset_version.sql y docs. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1167,7 +1252,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), **permanencia** acotada al rango: tabla de distribución con columna Acción (ojo por rango) que abre el listado de clientes de ese tramo; desde ahí ojo por cliente (volver al rango) y segundo ojito para asistencias por fecha/hora; **modal detalle permanencia: título con apellido y nombre** (junto al ID si aplica) cuando los datos lo permiten; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1266,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1548,9 +1633,20 @@
         <v>Se incorpora el apellido y nombre del cliente en el detalle de permanencia por cliente.</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>1.24</v>
+      </c>
+      <c r="B26" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Asistencia: RPC huella opcional (sql), cache sin re-fetch en sub-rango ni en refresh barra; modal rango ancho fit-content; ID+nombre en tabla clientes por bucket. everfit-release.json v1.24.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.25: gráfico activos asistencia, paginación 15k y último mes cerrado
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E51"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -942,7 +942,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -959,7 +959,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -976,7 +976,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -993,7 +993,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1010,7 +1010,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1027,7 +1027,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1044,7 +1044,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1061,7 +1061,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1078,7 +1078,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1095,7 +1095,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C41" t="str">
         <v>Despliegue v1.23</v>
@@ -1112,7 +1112,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C42" t="str">
         <v>Asistencia: huella RPC y cache</v>
@@ -1129,7 +1129,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C43" t="str">
         <v>Asistencia: refresh barra sin invalidar cache</v>
@@ -1146,7 +1146,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C44" t="str">
         <v>Asistencia: nombre en modal por rango</v>
@@ -1163,7 +1163,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C45" t="str">
         <v>Asistencia: sub-rango en memoria</v>
@@ -1180,7 +1180,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>14:03</v>
+        <v>16:08</v>
       </c>
       <c r="C46" t="str">
         <v>Despliegue v1.24</v>
@@ -1192,9 +1192,94 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B47" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Asistencia: gráfico activos + paginación 5000</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Card «Clientes activos por mes» (Chart.js líneas): mismos filtros que el mapa; activos = personas únicas con ingreso por mes calendario; MA3; Total+suavizado; varias sedes = línea por sede + tendencia total deduplicada; una sede = serie+suavizado. SUPABASE_PAGE_SIZE 5000 (alinear con Max rows en Supabase API).</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B48" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Paginación PostgREST: lotes reales + gráfico asistencia</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Asistencia: avanzar offset por filas devueltas y terminar con count exacto (evita cortar si Max rows &lt; pageSz; contador del modal = lotes reales). base_everfit y tipos de cambio: misma lógica hasta lote vacío. SUPABASE_PAGE_SIZE junto a createClient. Gráfico activos: resize doble rAF, min-height contenedor, iterar meses con guarda NaN.</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B49" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C49" t="str">
+        <v>SUPABASE_PAGE_SIZE 15000</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Constante en dashboard.html alineada con Max rows 15000 (Supabase Data API) para menos requests en base_everfit, tipos de cambio y transacciones_asistencia.</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B50" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Gráfico activos: hasta último mes cerrado</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Serie mensual cortada al último mes calendario completo en Argentina (excluye mes en curso); textos card y ayuda (?).</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B51" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Despliegue v1.25</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Asistencia: gráfico clientes activos/mes, paginación por lote real y SUPABASE_PAGE_SIZE 15000, eje hasta último mes cerrado AR; everfit-release.json y sidebar v1.25. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1252,7 +1337,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1351,7 +1436,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1644,9 +1729,20 @@
         <v>Asistencia: RPC huella opcional (sql), cache sin re-fetch en sub-rango ni en refresh barra; modal rango ancho fit-content; ID+nombre en tabla clientes por bucket. everfit-release.json v1.24.</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>1.25</v>
+      </c>
+      <c r="B27" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Asistencia: gráfico clientes activos por mes (MA3, filtros); paginación PostgREST por filas devueltas en base_everfit, tipos de cambio y asistencia; SUPABASE_PAGE_SIZE 15000; eje gráfico hasta último mes cerrado Argentina; everfit-release.json v1.25.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.26: modal nueva versión genérico (rendimiento servidor)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -942,7 +942,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -959,7 +959,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -976,7 +976,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -993,7 +993,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1010,7 +1010,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1027,7 +1027,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1044,7 +1044,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1061,7 +1061,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1078,7 +1078,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1095,7 +1095,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C41" t="str">
         <v>Despliegue v1.23</v>
@@ -1112,7 +1112,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C42" t="str">
         <v>Asistencia: huella RPC y cache</v>
@@ -1129,7 +1129,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C43" t="str">
         <v>Asistencia: refresh barra sin invalidar cache</v>
@@ -1146,7 +1146,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C44" t="str">
         <v>Asistencia: nombre en modal por rango</v>
@@ -1163,7 +1163,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C45" t="str">
         <v>Asistencia: sub-rango en memoria</v>
@@ -1180,7 +1180,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C46" t="str">
         <v>Despliegue v1.24</v>
@@ -1197,7 +1197,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C47" t="str">
         <v>Asistencia: gráfico activos + paginación 5000</v>
@@ -1214,7 +1214,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C48" t="str">
         <v>Paginación PostgREST: lotes reales + gráfico asistencia</v>
@@ -1231,7 +1231,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C49" t="str">
         <v>SUPABASE_PAGE_SIZE 15000</v>
@@ -1248,7 +1248,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C50" t="str">
         <v>Gráfico activos: hasta último mes cerrado</v>
@@ -1265,7 +1265,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>16:08</v>
+        <v>17:56</v>
       </c>
       <c r="C51" t="str">
         <v>Despliegue v1.25</v>
@@ -1277,9 +1277,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B52" t="str">
+        <v>17:56</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Gráfico activos: líneas multi-sede desde primer mes</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Con varias sucursales, cada serie usa null antes del primer mes con ≥1 activo en esa sede (evita tramo en cero antes de apertura). Textos card y ayuda (?).</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B53" t="str">
+        <v>17:56</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Despliegue v1.26</v>
+      </c>
+      <c r="D53" t="str">
+        <v>everfit-release.json: mensaje de nueva versión genérico (mejora tiempos de respuesta del servidor). Sidebar v1.26. Gráfico activos multi-sede desde primer mes con datos. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E53"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1337,7 +1371,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; con varias sedes cada línea arranca en el primer mes con datos de esa sede; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1436,7 +1470,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1740,9 +1774,20 @@
         <v>Asistencia: gráfico clientes activos por mes (MA3, filtros); paginación PostgREST por filas devueltas en base_everfit, tipos de cambio y asistencia; SUPABASE_PAGE_SIZE 15000; eje gráfico hasta último mes cerrado Argentina; everfit-release.json v1.25.</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>1.26</v>
+      </c>
+      <c r="B28" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Modal nueva versión: texto genérico orientado a tiempos de respuesta del servidor. Asistencia: líneas por sede en gráfico activos desde el primer mes con datos (sin ceros previos a la apertura). everfit-release.json v1.26.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.27: despliegue (modal genérico tiempos de respuesta)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -449,7 +449,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -466,7 +466,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -483,7 +483,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -500,7 +500,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -517,7 +517,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -534,7 +534,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -551,7 +551,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -568,7 +568,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -585,7 +585,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -602,7 +602,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -619,7 +619,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -636,7 +636,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -653,7 +653,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -670,7 +670,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -687,7 +687,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -704,7 +704,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -721,7 +721,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -738,7 +738,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -755,7 +755,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -772,7 +772,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -789,7 +789,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -806,7 +806,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -823,7 +823,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -840,7 +840,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -857,7 +857,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -874,7 +874,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -891,7 +891,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -908,7 +908,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -925,7 +925,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -942,7 +942,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -959,7 +959,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -976,7 +976,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -993,7 +993,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1010,7 +1010,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1027,7 +1027,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1044,7 +1044,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1061,7 +1061,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1078,7 +1078,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1095,7 +1095,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C41" t="str">
         <v>Despliegue v1.23</v>
@@ -1112,7 +1112,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C42" t="str">
         <v>Asistencia: huella RPC y cache</v>
@@ -1129,7 +1129,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C43" t="str">
         <v>Asistencia: refresh barra sin invalidar cache</v>
@@ -1146,7 +1146,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C44" t="str">
         <v>Asistencia: nombre en modal por rango</v>
@@ -1163,7 +1163,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C45" t="str">
         <v>Asistencia: sub-rango en memoria</v>
@@ -1180,7 +1180,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C46" t="str">
         <v>Despliegue v1.24</v>
@@ -1197,7 +1197,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C47" t="str">
         <v>Asistencia: gráfico activos + paginación 5000</v>
@@ -1214,7 +1214,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C48" t="str">
         <v>Paginación PostgREST: lotes reales + gráfico asistencia</v>
@@ -1231,7 +1231,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C49" t="str">
         <v>SUPABASE_PAGE_SIZE 15000</v>
@@ -1248,7 +1248,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C50" t="str">
         <v>Gráfico activos: hasta último mes cerrado</v>
@@ -1265,7 +1265,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C51" t="str">
         <v>Despliegue v1.25</v>
@@ -1282,7 +1282,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C52" t="str">
         <v>Gráfico activos: líneas multi-sede desde primer mes</v>
@@ -1299,7 +1299,7 @@
         <v>16/04/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>17:56</v>
+        <v>18:02</v>
       </c>
       <c r="C53" t="str">
         <v>Despliegue v1.26</v>
@@ -1311,9 +1311,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B54" t="str">
+        <v>18:02</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Gráfico activos: inicio por fecha mínima</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Null antes del primer mes con datos en total, una sede y cada línea multi-sede; MA3 sin tratar null como 0; tendencia total multi-sede recortada igual. Textos card y (?).</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="B55" t="str">
+        <v>18:02</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Despliegue v1.27</v>
+      </c>
+      <c r="D55" t="str">
+        <v>everfit-release.json: mensaje genérico (tiempos de respuesta del servidor). Sidebar v1.27. Gráfico activos: inicio por fecha mínima por sucursal/total y fix MA3 con null. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1371,7 +1405,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; con varias sedes cada línea arranca en el primer mes con datos de esa sede; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1470,7 +1504,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1785,9 +1819,20 @@
         <v>Modal nueva versión: texto genérico orientado a tiempos de respuesta del servidor. Asistencia: líneas por sede en gráfico activos desde el primer mes con datos (sin ceros previos a la apertura). everfit-release.json v1.26.</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>1.27</v>
+      </c>
+      <c r="B29" t="str">
+        <v>16/04/2026</v>
+      </c>
+      <c r="C29" t="str">
+        <v>everfit-release.json: aviso genérico de tiempos de respuesta. Gráfico activos: serie desde primer mes con datos (total, una o varias sedes); media móvil sin tratar null como cero.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.28: heatmap Promedio total y modal genérico
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -684,10 +684,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -701,10 +701,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -718,10 +718,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -735,10 +735,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -752,10 +752,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -769,10 +769,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -786,10 +786,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -803,10 +803,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -837,10 +837,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -854,10 +854,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -871,10 +871,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -888,10 +888,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -905,10 +905,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -922,10 +922,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -939,10 +939,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -956,10 +956,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -973,10 +973,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -990,10 +990,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1007,10 +1007,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1024,10 +1024,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1041,10 +1041,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1058,10 +1058,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1075,10 +1075,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1092,10 +1092,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C41" t="str">
         <v>Despliegue v1.23</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C42" t="str">
         <v>Asistencia: huella RPC y cache</v>
@@ -1126,10 +1126,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C43" t="str">
         <v>Asistencia: refresh barra sin invalidar cache</v>
@@ -1143,10 +1143,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C44" t="str">
         <v>Asistencia: nombre en modal por rango</v>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C45" t="str">
         <v>Asistencia: sub-rango en memoria</v>
@@ -1177,10 +1177,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C46" t="str">
         <v>Despliegue v1.24</v>
@@ -1194,10 +1194,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C47" t="str">
         <v>Asistencia: gráfico activos + paginación 5000</v>
@@ -1211,10 +1211,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C48" t="str">
         <v>Paginación PostgREST: lotes reales + gráfico asistencia</v>
@@ -1228,10 +1228,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C49" t="str">
         <v>SUPABASE_PAGE_SIZE 15000</v>
@@ -1245,10 +1245,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C50" t="str">
         <v>Gráfico activos: hasta último mes cerrado</v>
@@ -1262,10 +1262,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C51" t="str">
         <v>Despliegue v1.25</v>
@@ -1279,10 +1279,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C52" t="str">
         <v>Gráfico activos: líneas multi-sede desde primer mes</v>
@@ -1296,10 +1296,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C53" t="str">
         <v>Despliegue v1.26</v>
@@ -1313,10 +1313,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C54" t="str">
         <v>Gráfico activos: inicio por fecha mínima</v>
@@ -1330,24 +1330,58 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>18:02</v>
+        <v>09:41</v>
       </c>
       <c r="C55" t="str">
+        <v>Asistencia: fila Promedio total en heatmap</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Última fila del mapa de concurrencia = promedio aritmético por columna (hora) de las filas anteriores; maxVal incluye esa fila para misma escala de color; borde superior; leyenda.</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>17/04/2026</v>
+      </c>
+      <c r="B56" t="str">
+        <v>09:41</v>
+      </c>
+      <c r="C56" t="str">
         <v>Despliegue v1.27</v>
       </c>
-      <c r="D55" t="str">
+      <c r="D56" t="str">
         <v>everfit-release.json: mensaje genérico (tiempos de respuesta del servidor). Sidebar v1.27. Gráfico activos: inicio por fecha mínima por sucursal/total y fix MA3 con null. Push a main y vercel --prod.</v>
       </c>
-      <c r="E55" t="str">
+      <c r="E56" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>17/04/2026</v>
+      </c>
+      <c r="B57" t="str">
+        <v>09:41</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Despliegue v1.28</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Asistencia heatmap: fila «Promedio total» por hora (misma escala de color). everfit-release.json genérico. Sidebar v1.28. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E57" t="str">
         <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1405,7 +1439,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, **fila final «Promedio total»** por hora (promedio de las filas superiores, misma escala de color), años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1504,7 +1538,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1670,7 +1704,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
@@ -1681,7 +1715,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -1692,7 +1726,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Tipos de cambio con paginación al cargar (tipos_cambio_global / tipo_de_cambio). Regla proyecto: documentar límite PostgREST y paginación en reglas-everfit.</v>
@@ -1703,7 +1737,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Fechas America/Argentina/Buenos_Aires: gráfico G/P y clave mes en curso; fecha_pago ISO/timestamptz agrupada por día local (no slice UTC).</v>
@@ -1714,7 +1748,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Gráfico G/P Mensual alineado con tabla Flujo por mes (porMesFlujo; excluye Dividendos). Documentación EXCLUSIONES_DASHBOARD.md actualizada.</v>
@@ -1725,7 +1759,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Consolidado: fechas AR en agrupación y mes actual; gráfico=tabla Flujo; tarjetas con Dividendos; UX local sin anon key y errores sesión/RPC visibles. EXCLUSIONES_DASHBOARD.md.</v>
@@ -1736,7 +1770,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Asistencia: menú y permiso ver_asistencia (RLS, sql migración); heatmap por franja horaria, modo filas calendario o Lun–Dom, años vía RPC, optimización índice por fecha y caché; multi-sede con conteos por sede y lógica filtro una sede; UX carga filtros; índice (fecha,sucursal) en DDL.</v>
@@ -1747,7 +1781,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Asistencia frecuencia: distribución por rangos con días distintos ÷ semanas activas (lun–dom con ingreso); sin tramo &lt;1 día/sem.; prom. ingr./sem. activas en multi-sede; textos de ayuda.</v>
@@ -1758,7 +1792,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Asistencia: UX de carga (modal spinner y barra, área bajo filtros oculta hasta listo, progreso por descarga); aviso de muchos registros; modal «Nueva versión» con everfit-release.json (criterio Pandi); sql índice covering opcional; reglas bitácora y GIT_Y_VERCEL.</v>
@@ -1769,7 +1803,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Asistencia permanencia: columna Acción (ojo) por fila de rango abre modal con clientes de ese bucket; volver al rango desde el detalle; delegación de clics en document; sin tabla global detalle. everfit-release.json v1.22.</v>
@@ -1780,7 +1814,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Se incorpora el apellido y nombre del cliente en el detalle de permanencia por cliente.</v>
@@ -1791,7 +1825,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Asistencia: RPC huella opcional (sql), cache sin re-fetch en sub-rango ni en refresh barra; modal rango ancho fit-content; ID+nombre en tabla clientes por bucket. everfit-release.json v1.24.</v>
@@ -1802,7 +1836,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Asistencia: gráfico clientes activos por mes (MA3, filtros); paginación PostgREST por filas devueltas en base_everfit, tipos de cambio y asistencia; SUPABASE_PAGE_SIZE 15000; eje gráfico hasta último mes cerrado Argentina; everfit-release.json v1.25.</v>
@@ -1813,7 +1847,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Modal nueva versión: texto genérico orientado a tiempos de respuesta del servidor. Asistencia: líneas por sede en gráfico activos desde el primer mes con datos (sin ceros previos a la apertura). everfit-release.json v1.26.</v>
@@ -1824,15 +1858,26 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="C29" t="str">
         <v>everfit-release.json: aviso genérico de tiempos de respuesta. Gráfico activos: serie desde primer mes con datos (total, una o varias sedes); media móvil sin tratar null como cero.</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>1.28</v>
+      </c>
+      <c r="B30" t="str">
+        <v>17/04/2026</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Asistencia: fila final «Promedio total» en mapa de concurrencia (promedio por columna, misma escala de color). everfit-release.json v1.28 (mensaje genérico rendimiento).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.29: exclusión Flujo por concepto, proyección calendario y documentación
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E61"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C2" t="str">
         <v>Bitácora Everfit</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C3" t="str">
         <v>Despliegue v1.1</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C4" t="str">
         <v>Despliegue v1.2</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C5" t="str">
         <v>Despliegue v1.3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C6" t="str">
         <v>Despliegue v1.4</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C7" t="str">
         <v>Despliegue v1.5</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C8" t="str">
         <v>Despliegue v1.6</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C9" t="str">
         <v>Despliegue v1.7</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C10" t="str">
         <v>Despliegue v1.8</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C11" t="str">
         <v>Despliegue v1.9</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C12" t="str">
         <v>Despliegue v1.10</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C13" t="str">
         <v>Despliegue v1.11</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C14" t="str">
         <v>Despliegue v1.12</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C15" t="str">
         <v>Despliegue v1.13</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C16" t="str">
         <v>Despliegue v1.14</v>
@@ -684,10 +684,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C17" t="str">
         <v>Despliegue v1.15</v>
@@ -701,10 +701,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C18" t="str">
         <v>Dashboard fechas Argentina</v>
@@ -718,10 +718,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C19" t="str">
         <v>Despliegue v1.16</v>
@@ -735,10 +735,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C20" t="str">
         <v>Despliegue v1.17</v>
@@ -752,10 +752,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C21" t="str">
         <v>Dashboard local: mensaje si falta config</v>
@@ -769,10 +769,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C22" t="str">
         <v>Tarjetas: otra vez con Dividendos</v>
@@ -786,10 +786,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C23" t="str">
         <v>Despliegue v1.18</v>
@@ -803,10 +803,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C24" t="str">
         <v>Transacciones asistencia → Supabase</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C25" t="str">
         <v>Menú Asistencia en dashboard</v>
@@ -837,10 +837,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C26" t="str">
         <v>Combo año Asistencia desde datos</v>
@@ -854,10 +854,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C27" t="str">
         <v>Tabla multi-sede Asistencia</v>
@@ -871,10 +871,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C28" t="str">
         <v>Permiso ver_asistencia</v>
@@ -888,10 +888,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C29" t="str">
         <v>Despliegue v1.19</v>
@@ -905,10 +905,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: frecuencia de uso</v>
@@ -922,10 +922,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C31" t="str">
         <v>Despliegue v1.20</v>
@@ -939,10 +939,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C32" t="str">
         <v>Asistencia: permanencia</v>
@@ -956,10 +956,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C33" t="str">
         <v>Asistencia: permanencia aclaración</v>
@@ -973,10 +973,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C34" t="str">
         <v>Asistencia: filtros y rendimiento</v>
@@ -990,10 +990,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C35" t="str">
         <v>Asistencia: UX carga y SQL índice</v>
@@ -1007,10 +1007,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C36" t="str">
         <v>Nueva versión Everfit (como Pandi)</v>
@@ -1024,10 +1024,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C37" t="str">
         <v>Despliegue v1.21</v>
@@ -1041,10 +1041,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C38" t="str">
         <v>Asistencia: detalle permanencia por cliente</v>
@@ -1058,10 +1058,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C39" t="str">
         <v>Asistencia: permanencia ojo por rango</v>
@@ -1075,10 +1075,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C40" t="str">
         <v>Despliegue v1.22</v>
@@ -1092,10 +1092,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C41" t="str">
         <v>Despliegue v1.23</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C42" t="str">
         <v>Asistencia: huella RPC y cache</v>
@@ -1126,10 +1126,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C43" t="str">
         <v>Asistencia: refresh barra sin invalidar cache</v>
@@ -1143,10 +1143,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C44" t="str">
         <v>Asistencia: nombre en modal por rango</v>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C45" t="str">
         <v>Asistencia: sub-rango en memoria</v>
@@ -1177,10 +1177,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C46" t="str">
         <v>Despliegue v1.24</v>
@@ -1194,10 +1194,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C47" t="str">
         <v>Asistencia: gráfico activos + paginación 5000</v>
@@ -1211,10 +1211,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C48" t="str">
         <v>Paginación PostgREST: lotes reales + gráfico asistencia</v>
@@ -1228,10 +1228,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C49" t="str">
         <v>SUPABASE_PAGE_SIZE 15000</v>
@@ -1245,10 +1245,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C50" t="str">
         <v>Gráfico activos: hasta último mes cerrado</v>
@@ -1262,10 +1262,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C51" t="str">
         <v>Despliegue v1.25</v>
@@ -1279,10 +1279,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C52" t="str">
         <v>Gráfico activos: líneas multi-sede desde primer mes</v>
@@ -1296,10 +1296,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C53" t="str">
         <v>Despliegue v1.26</v>
@@ -1313,10 +1313,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C54" t="str">
         <v>Gráfico activos: inicio por fecha mínima</v>
@@ -1330,10 +1330,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C55" t="str">
         <v>Asistencia: fila Promedio total en heatmap</v>
@@ -1347,10 +1347,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C56" t="str">
         <v>Despliegue v1.27</v>
@@ -1364,10 +1364,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>09:41</v>
+        <v>08:53</v>
       </c>
       <c r="C57" t="str">
         <v>Despliegue v1.28</v>
@@ -1379,9 +1379,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>04/05/2026</v>
+      </c>
+      <c r="B58" t="str">
+        <v>08:53</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Flujo/GP: filtro por concepto</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Tabla Flujo y gráfico G/P excluyen filas con concepto Inversiones o Saldo Inicial (ya no por beneficiario Dividendos). Tarjetas y modal Detalle sin ese filtro por concepto. Ayudas (?) y docs/EXCLUSIONES_DASHBOARD.md actualizados.</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>04/05/2026</v>
+      </c>
+      <c r="B59" t="str">
+        <v>08:53</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Proyección: ventana calendario</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Base = N meses calendario anteriores al mes en curso (no últimos N con datos); relleno 0; ventana móvil Proy. 2+ con proyecciones previas. Modal y pie de tabla aclarados.</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>04/05/2026</v>
+      </c>
+      <c r="B60" t="str">
+        <v>08:53</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Proyección: documentación y blindaje</v>
+      </c>
+      <c r="D60" t="str">
+        <v>docs/PROYECCION_FLUJO.md; EXCLUSIONES y DASHBOARD actualizados. Código: filtro y lectura de montos solo para claves estrictamente anteriores al mes en curso (nunca mezclar mes en curso o futuros en la base).</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Documentación</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>04/05/2026</v>
+      </c>
+      <c r="B61" t="str">
+        <v>08:53</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Despliegue v1.29</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Flujo/G-P: exclusión por concepto Inversiones y Saldo Inicial; proyección con meses calendario previos al mes en curso y sin mes en curso/futuros en la base; docs PROYECCION_FLUJO, EXCLUSIONES, DASHBOARD; everfit-release.json v1.29. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1439,7 +1507,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen Dividendos (porMesFlujo); tarjetas totales incluyen todo salvo Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, **fila final «Promedio total»** por hora (promedio de las filas superiores, misma escala de color), años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen además concepto Inversiones y Saldo Inicial (porMesFlujo; no aplica a tarjetas ni Detalle); tarjetas totales incluyen todo salvo centro Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, **fila final «Promedio total»** por hora (promedio de las filas superiores, misma escala de color), años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1447,7 +1515,7 @@
         <v>Proyección Flujo por mes</v>
       </c>
       <c r="B7" t="str">
-        <v>Meses proyectados en tabla (permiso ver_proyeccion). Config: método (promedio/mediana/promedio recortado), meses de historia, meses a proyectar, recorte %. Ventana móvil. Total columna incluye proyectados; tarjetas siempre reales. Encabezado y celdas proyectadas con fondo distintivo.</v>
+        <v>Meses proyectados en tabla (permiso ver_proyeccion). Config: método (promedio/mediana/promedio recortado), meses de historia (N meses calendario estrictamente anteriores al mes en curso; nunca usa mes en curso ni futuros como base, aunque tengan datos), meses a proyectar, recorte %. Cada Proy. k usa los últimos (N−k) valores de esa ventana inicial más las k−1 proyecciones ya calculadas. Doc: docs/PROYECCION_FLUJO.md. Total columna incluye proyectados; tarjetas siempre reales. Encabezado y celdas proyectadas con fondo distintivo.</v>
       </c>
     </row>
     <row r="8">
@@ -1538,7 +1606,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1704,7 +1772,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtro multi-sucursal. Sucursales permitidas por usuario en Seguridad. Total respeta asignación. SQL supabase_sucursales_por_usuario.sql.</v>
@@ -1715,7 +1783,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -1726,7 +1794,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Tipos de cambio con paginación al cargar (tipos_cambio_global / tipo_de_cambio). Regla proyecto: documentar límite PostgREST y paginación en reglas-everfit.</v>
@@ -1737,7 +1805,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Fechas America/Argentina/Buenos_Aires: gráfico G/P y clave mes en curso; fecha_pago ISO/timestamptz agrupada por día local (no slice UTC).</v>
@@ -1748,7 +1816,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Gráfico G/P Mensual alineado con tabla Flujo por mes (porMesFlujo; excluye Dividendos). Documentación EXCLUSIONES_DASHBOARD.md actualizada.</v>
@@ -1759,7 +1827,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Consolidado: fechas AR en agrupación y mes actual; gráfico=tabla Flujo; tarjetas con Dividendos; UX local sin anon key y errores sesión/RPC visibles. EXCLUSIONES_DASHBOARD.md.</v>
@@ -1770,7 +1838,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Asistencia: menú y permiso ver_asistencia (RLS, sql migración); heatmap por franja horaria, modo filas calendario o Lun–Dom, años vía RPC, optimización índice por fecha y caché; multi-sede con conteos por sede y lógica filtro una sede; UX carga filtros; índice (fecha,sucursal) en DDL.</v>
@@ -1781,7 +1849,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Asistencia frecuencia: distribución por rangos con días distintos ÷ semanas activas (lun–dom con ingreso); sin tramo &lt;1 día/sem.; prom. ingr./sem. activas en multi-sede; textos de ayuda.</v>
@@ -1792,7 +1860,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Asistencia: UX de carga (modal spinner y barra, área bajo filtros oculta hasta listo, progreso por descarga); aviso de muchos registros; modal «Nueva versión» con everfit-release.json (criterio Pandi); sql índice covering opcional; reglas bitácora y GIT_Y_VERCEL.</v>
@@ -1803,7 +1871,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Asistencia permanencia: columna Acción (ojo) por fila de rango abre modal con clientes de ese bucket; volver al rango desde el detalle; delegación de clics en document; sin tabla global detalle. everfit-release.json v1.22.</v>
@@ -1814,7 +1882,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Se incorpora el apellido y nombre del cliente en el detalle de permanencia por cliente.</v>
@@ -1825,7 +1893,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Asistencia: RPC huella opcional (sql), cache sin re-fetch en sub-rango ni en refresh barra; modal rango ancho fit-content; ID+nombre en tabla clientes por bucket. everfit-release.json v1.24.</v>
@@ -1836,7 +1904,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Asistencia: gráfico clientes activos por mes (MA3, filtros); paginación PostgREST por filas devueltas en base_everfit, tipos de cambio y asistencia; SUPABASE_PAGE_SIZE 15000; eje gráfico hasta último mes cerrado Argentina; everfit-release.json v1.25.</v>
@@ -1847,7 +1915,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Modal nueva versión: texto genérico orientado a tiempos de respuesta del servidor. Asistencia: líneas por sede en gráfico activos desde el primer mes con datos (sin ceros previos a la apertura). everfit-release.json v1.26.</v>
@@ -1858,7 +1926,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C29" t="str">
         <v>everfit-release.json: aviso genérico de tiempos de respuesta. Gráfico activos: serie desde primer mes con datos (total, una o varias sedes); media móvil sin tratar null como cero.</v>
@@ -1869,15 +1937,26 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>17/04/2026</v>
+        <v>04/05/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Asistencia: fila final «Promedio total» en mapa de concurrencia (promedio por columna, misma escala de color). everfit-release.json v1.28 (mensaje genérico rendimiento).</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>1.29</v>
+      </c>
+      <c r="B31" t="str">
+        <v>04/05/2026</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Flujo/G-P exclusión concepto Inversiones y Saldo Inicial; proyección N meses calendario anteriores al mes en curso, blindaje mes en curso/futuros; docs PROYECCION_FLUJO.md y actualización EXCLUSIONES/DASHBOARD; everfit-release.json v1.29.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.30: To-Do bandeja, Sedes y mensajería interna
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E72"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1447,16 +1447,203 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B62" t="str">
+        <v>09:41</v>
+      </c>
+      <c r="C62" t="str">
+        <v>To-Do: módulo bandeja y roles</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Roles Recepcionista y Profesor; permisos ver_todo/crear_todo/completar_todo (alta por defecto Admin+Encargado); tablas todo_tarea/todo_instancia, RLS y RPCs; bandeja responsiva con filtros, estados, responsable obligatorio (usuario o perfil), recurrencias y export Excel. SQL helpers_fecha_argentina + supabase_todo; docs TODO/SEGURIDAD/DASHBOARD. Migración aplicada en Supabase Everfit.</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B63" t="str">
+        <v>09:53</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Sedes ABM + To-Do sede/fecha fin</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Menú Sedes (catálogo ABM) alimenta permisos por usuario y To-Do. Tareas: una sede o todas (réplica). Recurrentes exigen «hasta qué fecha» (máx. 366 días); se elimina la ventana fija de ~45 días. SQL supabase_sedes + supabase_todo_sede_y_fecha_fin; docs SEDES/TODO.</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B64" t="str">
+        <v>09:59</v>
+      </c>
+      <c r="C64" t="str">
+        <v>To-Do: fix read-only INSERT</v>
+      </c>
+      <c r="D64" t="str">
+        <v>todo_list_inbox ya no materializa instancias (STABLE/read-only en PostgREST). La generación va por todo_generar_instancias_todas antes del listado en el dashboard.</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B65" t="str">
+        <v>10:05</v>
+      </c>
+      <c r="C65" t="str">
+        <v>To-Do: bandeja no bloquea en generar</v>
+      </c>
+      <c r="D65" t="str">
+        <v>cargarTodoBandeja lista de inmediato; todo_generar_instancias_todas corre en background y refresca solo si creó instancias (evita quedar en «Cargando bandeja…»).</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B66" t="str">
+        <v>10:05</v>
+      </c>
+      <c r="C66" t="str">
+        <v>To-Do: editar/eliminar + vaciar prueba</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Permisos editar_todo y eliminar_todo (default Admin/Encargado, toggles en Seguridad). Modal editar y botón eliminar en bandeja. Tablas todo_tarea/todo_instancia vaciadas para prueba. SQL supabase_todo_editar_eliminar.sql.</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B67" t="str">
+        <v>10:11</v>
+      </c>
+      <c r="C67" t="str">
+        <v>To-Do: recurrencias bimestral/trimestral</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Se elimina hora_fija (igual que diaria con hora). Se agregan bimestral y trimestral. SQL constraints + todo_next_dates + UI.</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B68" t="str">
+        <v>10:13</v>
+      </c>
+      <c r="C68" t="str">
+        <v>To-Do: cards según filtros + Hoy default</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Las cards de resumen se calculan sobre el listado filtrado (estado/prioridad/vencimiento/sede/búsqueda). Filtro de vencimiento por defecto: Hoy.</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B69" t="str">
+        <v>14:43</v>
+      </c>
+      <c r="C69" t="str">
+        <v>To-Do: celdas centradas verticalmente</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Tabla de bandeja: vertical-align middle en td para alinear texto/badges con la fila de acciones (select + editar/eliminar).</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B70" t="str">
+        <v>14:43</v>
+      </c>
+      <c r="C70" t="str">
+        <v>To-Do: solapas Tareas + Por responsable</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Bandeja en solapa Tareas. Nueva solapa Por responsable (solo Admin/Encargado): matriz responsable×estado con los mismos filtros; clic en cantidad abre modal con el detalle de tareas.</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B71" t="str">
+        <v>15:03</v>
+      </c>
+      <c r="C71" t="str">
+        <v>To-Do: fix eliminar + mensajes + Empresa</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Eliminar ya no regenera la instancia (cancelada / desactiva plantilla). Mensajería estilo Pandi (toast + confirm). Alta con opción Empresa (una sola tarea sin sede). SQL supabase_todo_empresa_y_eliminar.sql.</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B72" t="str">
+        <v>19:50</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Despliegue v1.30</v>
+      </c>
+      <c r="D72" t="str">
+        <v>To-Do: bandeja, solapas Tareas/Por responsable, sede Empresa, eliminar sin regenerar, mensajería interna, alineación Tarea/Sede/Responsable. Menú Sedes. everfit-release.json v1.30. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E72"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1523,7 +1710,7 @@
         <v>Seguridad – Permisos por rol</v>
       </c>
       <c r="B8" t="str">
-        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Visor) con icono y lista de permisos con toggle on/off editable (incluye ver_asistencia para el menú Asistencia). RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql y sql/supabase_asistencia_ver_permiso.sql si aplica.</v>
+        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Recepcionista, Profesor, Visor) con icono y lista de permisos con toggle on/off editable (incluye ver_asistencia y permisos To-Do). RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql, sql/supabase_asistencia_ver_permiso.sql y sql/supabase_todo.sql si aplica.</v>
       </c>
     </row>
     <row r="9">
@@ -1534,9 +1721,25 @@
         <v>Excel export Transacciones por sucursal (docs de referencia). Tabla transacciones_asistencia; botón Importar asistencia en dashboard (reemplazo por sucursal). Ver docs/TRANSACCIONES_ASISTENCIA.md y sql/supabase_transacciones_asistencia.sql.</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>To-Do – bandeja de tareas</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; vencimiento por defecto Hoy), filtros (estado/prioridad/vencimiento/sede/búsqueda), badges, cambio de estado, alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con fecha «hasta» obligatoria (máx. 366 días), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Sedes – catálogo ABM</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1606,7 +1809,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1954,9 +2157,20 @@
         <v>Flujo/G-P exclusión concepto Inversiones y Saldo Inicial; proyección N meses calendario anteriores al mes en curso, blindaje mes en curso/futuros; docs PROYECCION_FLUJO.md y actualización EXCLUSIONES/DASHBOARD; everfit-release.json v1.29.</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>1.30</v>
+      </c>
+      <c r="B32" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="C32" t="str">
+        <v>To-Do (bandeja, filtros Hoy, solapas Tareas y Por responsable, alta Empresa/sede, eliminar sin regenerar, toast/confirm). Catálogo Sedes. Roles Recepcionista/Profesor. everfit-release.json v1.30.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.31: Configuración reasignar To-Do, filtros abiertas y resalte activo
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E76"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1634,16 +1634,84 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B73" t="str">
+        <v>20:12</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Configuración: reasignar To-Do</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Menú Configuración (permiso ver_configuracion, Admin/Encargado). Reasignar una, varias o todas las tareas abiertas de un usuario a otro o de un perfil a otro. SQL supabase_todo_reasignar.sql; docs CONFIGURACION.</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B74" t="str">
+        <v>20:26</v>
+      </c>
+      <c r="C74" t="str">
+        <v>To-Do: filtro estado Abiertas por defecto</v>
+      </c>
+      <c r="D74" t="str">
+        <v>El filtro de estado inicia en Abiertas (pendiente, en curso y vencida). Hechas y canceladas no se listan hasta que se elijan. Al filtrar Hecha/Cancelada con vencimiento Hoy, el vencimiento pasa a Todas para poder reabrir. SQL supabase_todo_inbox_estado_abiertas.sql.</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B75" t="str">
+        <v>20:33</v>
+      </c>
+      <c r="C75" t="str">
+        <v>To-Do: resaltar filtros activos</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Los filtros que recortan la bandeja (estado distinto de Todos, vencimiento distinto de Todas, prioridad, sede o búsqueda) se marcan con estilo activo y leyenda «activo».</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B76" t="str">
+        <v>20:59</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Despliegue v1.31</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Menú Configuración (reasignar To-Do por usuario o perfil). To-Do: estado Abiertas por defecto y resalte de filtros activos. everfit-release.json v1.31. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E76"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1726,7 +1794,7 @@
         <v>To-Do – bandeja de tareas</v>
       </c>
       <c r="B10" t="str">
-        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; vencimiento por defecto Hoy), filtros (estado/prioridad/vencimiento/sede/búsqueda), badges, cambio de estado, alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con fecha «hasta» obligatoria (máx. 366 días), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql.</v>
+        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; estado por defecto Abiertas = pendiente/en curso/vencida; vencimiento por defecto Hoy), filtros resaltados cuando recortan el listado (estado/prioridad/vencimiento/sede/búsqueda), badges, cambio de estado, alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con fecha «hasta» obligatoria (máx. 366 días), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql.</v>
       </c>
     </row>
     <row r="11">
@@ -1737,9 +1805,17 @@
         <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Configuración – reasignar To-Do</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Menú Configuración (permiso ver_configuracion, default Admin/Encargado). Reasignar una, varias o todas las tareas abiertas de un usuario a otro, o de un perfil a otro (p. ej. Recepcionista → Profesor). SQL: sql/supabase_todo_reasignar.sql. Docs: docs/CONFIGURACION.md.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1809,7 +1885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2168,9 +2244,20 @@
         <v>To-Do (bandeja, filtros Hoy, solapas Tareas y Por responsable, alta Empresa/sede, eliminar sin regenerar, toast/confirm). Catálogo Sedes. Roles Recepcionista/Profesor. everfit-release.json v1.30.</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>1.31</v>
+      </c>
+      <c r="B33" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Menú Configuración: reasignar tareas To-Do de un usuario a otro o de un perfil a otro. To-Do: filtro estado Abiertas por defecto y resalte de filtros activos. everfit-release.json v1.31.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.32: primer vencimiento en tareas recurrentes
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E78"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1702,9 +1702,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B77" t="str">
+        <v>21:12</v>
+      </c>
+      <c r="C77" t="str">
+        <v>To-Do: primer vencimiento de la serie</v>
+      </c>
+      <c r="D77" t="str">
+        <v>En recurrentes se elige el primer due date (p. ej. el lunes próximo) y desde ahí se replica: diario +1, semanal +7, trimestral +3 meses, etc. Se ocultan día de semana / día del mes. SQL supabase_todo_primer_vencimiento.sql.</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B78" t="str">
+        <v>21:13</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Despliegue v1.32</v>
+      </c>
+      <c r="D78" t="str">
+        <v>To-Do recurrente: primer vencimiento a elección y réplica de la serie desde esa fecha. everfit-release.json v1.32. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E78"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1794,7 +1828,7 @@
         <v>To-Do – bandeja de tareas</v>
       </c>
       <c r="B10" t="str">
-        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; estado por defecto Abiertas = pendiente/en curso/vencida; vencimiento por defecto Hoy), filtros resaltados cuando recortan el listado (estado/prioridad/vencimiento/sede/búsqueda), badges, cambio de estado, alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con fecha «hasta» obligatoria (máx. 366 días), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql.</v>
+        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; estado por defecto Abiertas = pendiente/en curso/vencida; vencimiento por defecto Hoy), filtros resaltados cuando recortan el listado, badges, cambio de estado, alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql + supabase_todo_primer_vencimiento.sql.</v>
       </c>
     </row>
     <row r="11">
@@ -1885,7 +1919,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2255,9 +2289,20 @@
         <v>Menú Configuración: reasignar tareas To-Do de un usuario a otro o de un perfil a otro. To-Do: filtro estado Abiertas por defecto y resalte de filtros activos. everfit-release.json v1.31.</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>1.32</v>
+      </c>
+      <c r="B34" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="C34" t="str">
+        <v>To-Do recurrente: se indica el primer vencimiento y desde ahí se replica la serie (diario, semanal, trimestral, etc.). everfit-release.json v1.32.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.33: en curso en cards y sin vencimientos domingo
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E80"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1736,9 +1736,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B79" t="str">
+        <v>21:21</v>
+      </c>
+      <c r="C79" t="str">
+        <v>To-Do: en curso + sin domingo</v>
+      </c>
+      <c r="D79" t="str">
+        <v>En curso se cuenta en cards y Por responsable aunque esté vencida la fecha. No se registran tareas en domingo (AR): diaria omite el día; mensual/trimestral pasa al lunes. SQL supabase_todo_en_curso_sin_domingo.sql.</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="B80" t="str">
+        <v>21:22</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Despliegue v1.33</v>
+      </c>
+      <c r="D80" t="str">
+        <v>To-Do: en curso se cuenta aunque esté vencida la fecha; sin vencimientos en domingo. everfit-release.json v1.33. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E80"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1919,7 +1953,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2300,9 +2334,20 @@
         <v>To-Do recurrente: se indica el primer vencimiento y desde ahí se replica la serie (diario, semanal, trimestral, etc.). everfit-release.json v1.32.</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>1.33</v>
+      </c>
+      <c r="B35" t="str">
+        <v>13/08/2026</v>
+      </c>
+      <c r="C35" t="str">
+        <v>To-Do: en curso se cuenta en cards y Por responsable aunque esté vencida la fecha; no se registran vencimientos en domingo. everfit-release.json v1.33.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.34: diaria Hecha recién al vencimiento
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E82"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1770,9 +1770,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>14/08/2026</v>
+      </c>
+      <c r="B81" t="str">
+        <v>09:33</v>
+      </c>
+      <c r="C81" t="str">
+        <v>To-Do: diaria Hecha al vencer</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Una tarea con recurrencia diaria no se puede marcar Hecha antes de su vencimiento (control en bandeja y en todo_cambiar_estado). SQL supabase_todo_diaria_hecha_al_vencer.sql.</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>14/08/2026</v>
+      </c>
+      <c r="B82" t="str">
+        <v>18:15</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Despliegue v1.34</v>
+      </c>
+      <c r="D82" t="str">
+        <v>To-Do: las diarias no se marcan Hecha antes del vencimiento. everfit-release.json v1.34. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E82"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1862,7 +1896,7 @@
         <v>To-Do – bandeja de tareas</v>
       </c>
       <c r="B10" t="str">
-        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; estado por defecto Abiertas = pendiente/en curso/vencida; vencimiento por defecto Hoy), filtros resaltados cuando recortan el listado, badges, cambio de estado, alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql + supabase_todo_primer_vencimiento.sql.</v>
+        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; estado por defecto Abiertas = pendiente/en curso/vencida; vencimiento por defecto Hoy), filtros resaltados cuando recortan el listado, badges, cambio de estado (diaria: Hecha recién al vencimiento), alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date; sin domingos), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql + supabase_todo_primer_vencimiento.sql + supabase_todo_en_curso_sin_domingo.sql + supabase_todo_diaria_hecha_al_vencer.sql.</v>
       </c>
     </row>
     <row r="11">
@@ -1953,7 +1987,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2345,9 +2379,20 @@
         <v>To-Do: en curso se cuenta en cards y Por responsable aunque esté vencida la fecha; no se registran vencimientos en domingo. everfit-release.json v1.33.</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>1.34</v>
+      </c>
+      <c r="B36" t="str">
+        <v>14/08/2026</v>
+      </c>
+      <c r="C36" t="str">
+        <v>To-Do: una tarea diaria no se puede marcar Hecha antes de su vencimiento. everfit-release.json v1.34.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.35: To-Do Hecha el mismo día y card Hechas hoy
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E85"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1804,9 +1804,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B83" t="str">
+        <v>14:34</v>
+      </c>
+      <c r="C83" t="str">
+        <v>To-Do: diaria Hecha el mismo día</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Diaria: se puede marcar Hecha en cualquier hora del día de vencimiento (Argentina); solo se bloquea si el vencimiento es un día posterior a hoy. Bandeja + todo_cambiar_estado. SQL supabase_todo_diaria_hecha_mismo_dia.sql.</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B84" t="str">
+        <v>14:38</v>
+      </c>
+      <c r="C84" t="str">
+        <v>To-Do: card Hechas hoy</v>
+      </c>
+      <c r="D84" t="str">
+        <v>La card Hechas hoy ya no sale del listado Abiertas (quedaba en 0). RPC todo_list_hechas_hoy por día calendario AR, sin recorte por hora. Respeta sede, prioridad y búsqueda.</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Corrección</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B85" t="str">
+        <v>14:48</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Despliegue v1.35</v>
+      </c>
+      <c r="D85" t="str">
+        <v>To-Do: diaria Hecha el mismo día (sin hora límite); card Hechas hoy independiente del filtro Abiertas. everfit-release.json v1.35. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E85"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1896,7 +1947,7 @@
         <v>To-Do – bandeja de tareas</v>
       </c>
       <c r="B10" t="str">
-        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (cards según filtros; estado por defecto Abiertas = pendiente/en curso/vencida; vencimiento por defecto Hoy), filtros resaltados cuando recortan el listado, badges, cambio de estado (diaria: Hecha recién al vencimiento), alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date; sin domingos), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql + supabase_todo_primer_vencimiento.sql + supabase_todo_en_curso_sin_domingo.sql + supabase_todo_diaria_hecha_al_vencer.sql.</v>
+        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (Pendientes/En curso/Vencidas según listado; Hechas hoy por día calendario aunque el filtro sea Abiertas), filtros resaltados cuando recortan el listado, badges, cambio de estado (diaria: Hecha el mismo día de vencimiento, sin exigir la hora), alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date; sin domingos), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql + supabase_todo_primer_vencimiento.sql + supabase_todo_en_curso_sin_domingo.sql + supabase_todo_diaria_hecha_al_vencer.sql + supabase_todo_diaria_hecha_mismo_dia.sql + supabase_todo_hechas_hoy.sql.</v>
       </c>
     </row>
     <row r="11">
@@ -1987,7 +2038,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2390,9 +2441,20 @@
         <v>To-Do: una tarea diaria no se puede marcar Hecha antes de su vencimiento. everfit-release.json v1.34.</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>1.35</v>
+      </c>
+      <c r="B37" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="C37" t="str">
+        <v>To-Do: diaria se marca Hecha el mismo día de vencimiento (sin esperar la hora); card Hechas hoy se actualiza con Abiertas. everfit-release.json v1.35.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.36: To-Do perfil, Usuario, menús por rol y bandeja móvil
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E92"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1855,9 +1855,128 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B86" t="str">
+        <v>19:23</v>
+      </c>
+      <c r="C86" t="str">
+        <v>To-Do: modal responsive</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Modales nueva/editar tarea: cuerpo con scroll, footer fijo con botones visibles en PC y móvil (safe-area, 768px).</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B87" t="str">
+        <v>19:23</v>
+      </c>
+      <c r="C87" t="str">
+        <v>To-Do: columna Estado por</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Bandeja, matriz y Excel muestran quién cambió el estado por última vez. Columna todo_instancia.estado_modificado_por; todo_cambiar_estado y todo_list_inbox. SQL supabase_todo_estado_modificado_por.sql.</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B88" t="str">
+        <v>19:23</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Permiso ver_dashboard</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Menú Home (Dashboard) configurable por rol en Seguridad, igual que Asistencia (ver_asistencia). Vista inicial según permisos. SQL supabase_menu_ver_dashboard.sql.</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B89" t="str">
+        <v>19:30</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Mi perfil: nombre de usuario</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Columna nombre_usuario en user_profiles; modal Mi perfil en barra superior; bandeja To-Do (Responsable y Usuario) y combos usan nombre en lugar de email. RPC get_my_profile, set_my_nombre_usuario, user_profile_label. SQL supabase_user_profiles_nombre_usuario.sql.</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B90" t="str">
+        <v>19:42</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Seguridad: editar nombre usuario</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Tabla Usuarios con email + campo Nombre para mostrar; Guardar persiste rol y nombre (RPC set_user_nombre_usuario). Columna bandeja To-Do renombrada a Usuario. SQL supabase_set_user_nombre_usuario_admin.sql.</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B91" t="str">
+        <v>19:46</v>
+      </c>
+      <c r="C91" t="str">
+        <v>To-Do: tabla mobile</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Bandeja: columnas auto (max-content), scroll horizontal; Acción 4.ª columna; Tarea y Acción sticky en scroll móvil.</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B92" t="str">
+        <v>19:46</v>
+      </c>
+      <c r="C92" t="str">
+        <v>To-Do: tooltip email</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Responsable y Usuario: hover/tap muestra email flotante con botón Copiar; RPC todo_list_inbox devuelve responsable_email y estado_modificado_email. SQL supabase_todo_list_inbox_emails.sql.</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E92"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1915,7 +2034,7 @@
         <v>Dashboard Everfit</v>
       </c>
       <c r="B6" t="str">
-        <v>Una página (dashboard.html): flujo por mes y gráfico G/P excluyen además concepto Inversiones y Saldo Inicial (porMesFlujo; no aplica a tarjetas ni Detalle); tarjetas totales incluyen todo salvo centro Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, **fila final «Promedio total»** por hora (promedio de las filas superiores, misma escala de color), años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
+        <v>Una página (dashboard.html): menú Home (permiso ver_dashboard, configurable en Seguridad). Flujo por mes y gráfico G/P excluyen además concepto Inversiones y Saldo Inicial (porMesFlujo; no aplica a tarjetas ni Detalle); tarjetas totales incluyen todo salvo centro Saldo Inicial (porMes). Importar asistencia (Excel → transacciones_asistencia, upload_base). Menú Asistencia (permiso ver_asistencia): heatmap por concurrencia (colores, franja horaria), filas calendario o Lun–Dom, **fila final «Promedio total»** por hora (promedio de las filas superiores, misma escala de color), años con datos (RPC) y opción «Todos los años», mes «Todos los meses» por defecto al entrar o al abrir importar; filtro sucursal con delegación de clic; vista activa por ítem de menú; mapa y métricas escalonados (rAF). **Gráfico clientes activos por mes** (personas únicas con ingreso por mes calendario, eje hasta último mes cerrado AR, MA3; cada serie desde el primer mes con datos de su contexto—total, una sede o cada sede—sin ceros previos; total / varias sedes / una sede según filtro). Carga de transacciones: área bajo filtros en blanco, modal con spinner y barra de progreso (count + páginas), fase de armado del mapa; **RPC opcional get_asistencia_dataset_version**; **sub-rango del combo filtrado en memoria** si el rectángulo ya está descargado; **Actualizar permisos (barra) no invalida** el cache de asistencia; índice covering opcional en sql/. Paginación PostgREST **SUPABASE_PAGE_SIZE 15000** (coherente con Max rows del proyecto en Supabase Data API). Frecuencia (días distintos ÷ semanas activas), **permanencia**: ojo por rango, **modal listado clientes** ancho según contenido e **ID — apellido y nombre** en tabla; modal detalle con título apellido/nombre; multi-sede. Tras un despliegue: modal «Nueva versión» (**everfit-release.json**). Fechas America/Argentina/Buenos_Aires. Login; Seguridad; actualizar base; carga paginada base_everfit, tipos de cambio y asistencia por rango.</v>
       </c>
     </row>
     <row r="7">
@@ -1931,7 +2050,7 @@
         <v>Seguridad – Permisos por rol</v>
       </c>
       <c r="B8" t="str">
-        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Recepcionista, Profesor, Visor) con icono y lista de permisos con toggle on/off editable (incluye ver_asistencia y permisos To-Do). RPC get_roles_permissions_for_admin y set_role_permission. Ejecutar sql/supabase_seguridad_permisos_editable.sql, sql/supabase_asistencia_ver_permiso.sql y sql/supabase_todo.sql si aplica.</v>
+        <v>En Seguridad (Admin): cada rol (Admin, Encargado, Recepcionista, Profesor, Visor) con icono y lista de permisos con toggle on/off editable (incluye ver_dashboard, ver_asistencia y permisos To-Do). Tabla Usuarios: email, nombre para mostrar (editable), rol y sucursales. RPC get_roles_permissions_for_admin, set_role_permission y set_user_nombre_usuario. Ejecutar sql/supabase_seguridad_permisos_editable.sql, sql/supabase_menu_ver_dashboard.sql, sql/supabase_asistencia_ver_permiso.sql, sql/supabase_user_profiles_nombre_usuario.sql y sql/supabase_set_user_nombre_usuario_admin.sql si aplica.</v>
       </c>
     </row>
     <row r="9">
@@ -1947,7 +2066,7 @@
         <v>To-Do – bandeja de tareas</v>
       </c>
       <c r="B10" t="str">
-        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Resumen (Pendientes/En curso/Vencidas según listado; Hechas hoy por día calendario aunque el filtro sea Abiertas), filtros resaltados cuando recortan el listado, badges, cambio de estado (diaria: Hecha el mismo día de vencimiento, sin exigir la hora), alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date; sin domingos), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + supabase_todo_sede_y_fecha_fin.sql + supabase_todo_editar_eliminar.sql + supabase_todo_empresa_y_eliminar.sql + supabase_todo_inbox_estado_abiertas.sql + supabase_todo_primer_vencimiento.sql + supabase_todo_en_curso_sin_domingo.sql + supabase_todo_diaria_hecha_al_vencer.sql + supabase_todo_diaria_hecha_mismo_dia.sql + supabase_todo_hechas_hoy.sql.</v>
+        <v>Menú To-Do: solapas Tareas y Por responsable (Admin/Encargado: matriz perfil/usuario × estado con clic a modal de detalle). Columna **Usuario** (nombre de quien cambió el estado por última vez; sin email en bandeja). **Mi perfil** o **Seguridad → Usuarios**: nombre para mostrar. Modales nueva/editar con scroll y footer fijo en móvil. Resumen (Pendientes/En curso/Vencidas según listado; Hechas hoy por día calendario aunque el filtro sea Abiertas), filtros resaltados cuando recortan el listado, badges, cambio de estado (diaria: Hecha el mismo día de vencimiento, sin exigir la hora), alta con responsable obligatorio (usuario o perfil), sede (una / todas / Empresa), recurrencia con primer vencimiento + «hasta» (máx. 366 días; la serie se replica desde ese due date; sin domingos), editar/eliminar (sin regenerar), mensajería interna toast/confirm, export Excel. Permisos ver_todo/crear_todo/completar_todo/editar_todo/eliminar_todo. Roles Recepcionista y Profesor. Docs: docs/TODO.md; SQL: sql/supabase_todo.sql + … + supabase_user_profiles_nombre_usuario.sql + supabase_set_user_nombre_usuario_admin.sql.</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
v1.37: fix scroll To-Do en celular vertical
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E94"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1974,9 +1974,43 @@
         <v>Feature</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B93" t="str">
+        <v>19:54</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Despliegue v1.36</v>
+      </c>
+      <c r="D93" t="str">
+        <v>To-Do: Mi perfil y nombre visible; columna Usuario; tooltip email copiar; bandeja mobile (Acción 4.ª); modales responsive; ver_dashboard y nombres en Seguridad. everfit-release.json v1.36. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B94" t="str">
+        <v>19:57</v>
+      </c>
+      <c r="C94" t="str">
+        <v>To-Do: scroll móvil vertical</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Bandeja: en portrait la tabla se cortaba en la 4.ª columna (Acción sticky + min-width 100%). Sin sticky Acción en ≤768px, scroll horizontal en el wrap, hint deslizar, main-content sin overflow-x.</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Fix</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E94"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2157,7 +2191,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2571,9 +2605,20 @@
         <v>To-Do: diaria se marca Hecha el mismo día de vencimiento (sin esperar la hora); card Hechas hoy se actualiza con Abiertas. everfit-release.json v1.35.</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>1.36</v>
+      </c>
+      <c r="B38" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="C38" t="str">
+        <v>To-Do: Mi perfil (nombre para mostrar); columna Usuario; tooltip email copiar en Responsable/Usuario; bandeja mobile (Acción 4.ª, scroll horizontal); modales nueva/editar responsive; permiso ver_dashboard; Seguridad edita nombre por usuario. SQL migraciones Supabase. everfit-release.json v1.36.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>